<commit_message>
Breaking Changes: - Workbook_GetWorksheet: Output Paramater Change.
New Function:
- Image_Get: Get Image from the Spreadsheet
- Image_GetAll_InCell: Get All Images (In Cell Only) from the Spreadsheet
- Image_GetAll_OverCell: Get All Images (Over Cell Only) from the Spreadsheet
- Range_FromAddress: Convert Given Address to the Cell Range format
- Worksheet_Copy: Copy Worksheet from another Excel File
- Worksheet_GetProperties: Get All Worksheets Properties in the Spreadsheet

New Update:
- Update EPPlus version 8.0.5

Limitation:
- The default image upload in the Excel spreadsheet is set to 'Over Cell'. To get an image 'In Cell', a separate function is needed starting from EPPlus 8 onward.
</commit_message>
<xml_diff>
--- a/Result/MergeResult.xlsx
+++ b/Result/MergeResult.xlsx
@@ -12,8 +12,16 @@
     <sheet name="Sheet3C" sheetId="5" r:id="rId5"/>
     <sheet name="Sheet4" sheetId="6" r:id="rId6"/>
     <sheet name="Sheet1-2" sheetId="7" r:id="rId7"/>
+    <sheet name="Sheet1-3" sheetId="8" r:id="rId9"/>
+    <sheet name="Sheet2-2" sheetId="9" r:id="rId10"/>
+    <sheet name="Sheet3C-1" sheetId="10" r:id="rId11"/>
+    <sheet name="Sheet4-1" sheetId="11" r:id="rId12"/>
+    <sheet name="Sheet1-4" sheetId="12" r:id="rId13"/>
+    <sheet name="Sheet2-3" sheetId="13" r:id="rId14"/>
+    <sheet name="Sheet3C-2" sheetId="14" r:id="rId15"/>
+    <sheet name="Sheet4-2" sheetId="15" r:id="rId16"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr fullCalcOnLoad="1" fullPrecision="1"/>
 </workbook>
 </file>
 
@@ -85,7 +93,7 @@
   <fonts count="1">
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="2">
@@ -140,8 +148,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F655E9FF-620C-0F4B-911F-DED93BAAB0B0}">
-  <sheetPr codeName=""/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C3C9297-22D8-494D-B179-69EBE75E586F}">
   <dimension ref="B3:E16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -166,9 +173,159 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06E9A583-CFF2-4C3A-B002-55C1D9A31125}">
+  <sheetPr>
+    <tabColor rgb="FF3B7D23"/>
+  </sheetPr>
+  <dimension ref="AA5:AA8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="5">
+      <c r="AA5" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="AA6" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="AA7" s="0">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="AA8" s="0">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20455092-0F4C-4524-96E6-967C17E5509C}">
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1188BBB1-2206-40EF-9E54-65ACD4069337}">
+  <sheetPr>
+    <tabColor rgb="FFC04F15"/>
+  </sheetPr>
+  <dimension ref="A5:A9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7DDDEDD-EFA8-4D6D-84FE-EEE6F3277DAC}">
+  <dimension ref="J6:J8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="6">
+      <c r="J6" s="0" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="J7" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="J8" s="0" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD3DB106-7900-4EDB-AF8D-B27C3B068FEB}">
+  <sheetPr>
+    <tabColor rgb="FF3B7D23"/>
+  </sheetPr>
+  <dimension ref="AA5:AA8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="5">
+      <c r="AA5" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="AA6" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="AA7" s="0">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="AA8" s="0">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1D6648C-2890-4547-B493-D1E730E6B18D}">
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8485F015-C74F-484A-AAA9-5644054DD2EE}">
-  <sheetPr codeName=""/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2832CA2-D306-4D2C-86D5-4FEC24176947}">
   <dimension ref="B3:C208"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -189,9 +346,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{817EA029-6624-EF44-8FC8-3C7BDF15A6FE}">
-  <sheetPr codeName="">
-    <tabColor theme="5" tint="-0.249977111117893"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A82A55CF-53B8-499A-A567-BC0F5F85E881}">
+  <sheetPr>
+    <tabColor rgb="FFC04F15"/>
   </sheetPr>
   <dimension ref="A5:A9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -228,8 +385,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04223B19-F040-F942-AA10-32B980D184CC}">
-  <sheetPr codeName=""/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29BE7371-A158-44A8-B498-3A5F8D78E960}">
   <dimension ref="J6:J8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -255,9 +411,9 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B62E063-A667-104D-AD79-2B258367AAD4}">
-  <sheetPr codeName="">
-    <tabColor theme="9" tint="-0.249977111117893"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AF7863A-C664-42AC-9051-FC6D217F1133}">
+  <sheetPr>
+    <tabColor rgb="FF3B7D23"/>
   </sheetPr>
   <dimension ref="AA5:AA8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -289,8 +445,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83775252-BBA6-4E40-80AD-84532B55B83D}">
-  <sheetPr codeName=""/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B746711-C1A5-4C99-B52D-1147AD3F44D3}">
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -299,8 +454,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1A6D69B-B770-224B-8690-C75033EFA29B}">
-  <sheetPr codeName=""/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D16284C-8DBE-487F-A9B1-57FF67877C45}">
   <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -346,7 +500,6 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="B3" s="0">
         <v>1</v>
@@ -368,33 +521,21 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="G8" s="0" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="G10" s="0" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="G12" s="0" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
@@ -402,4 +543,74 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC91033E-695E-49F8-83DC-56284E2D9D3B}">
+  <sheetPr>
+    <tabColor rgb="FFC04F15"/>
+  </sheetPr>
+  <dimension ref="A5:A9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EA38CA4-28C3-4A84-A350-2B02DBDF2C52}">
+  <dimension ref="J6:J8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="6">
+      <c r="J6" s="0" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="J7" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="J8" s="0" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=EPPlusLicense.txt>This workbook was created with the EPPlus library, licensed to OutSystems Community under the Polyform Noncommercial license, see https://polyformproject.org/licenses/noncommercial/1.0.0
+For more information about EPPlus, see https://epplussoftware.com/
+
 </file>
</xml_diff>